<commit_message>
Updated Excel file via Streamlit
</commit_message>
<xml_diff>
--- a/Pharma_Society_Report.xlsx
+++ b/Pharma_Society_Report.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
   <si>
     <t>Society Name</t>
   </si>
@@ -62,21 +62,6 @@
   </si>
   <si>
     <t>MOASC (Medical Oncology Association of Southern California)</t>
-  </si>
-  <si>
-    <t>600</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>176</t>
-  </si>
-  <si>
-    <t>400</t>
   </si>
   <si>
     <t>No, FLASCO does not encompass community sites, FLASCO's membership primarily consists of academic and hospital-based oncologists and hematologists.</t>
@@ -610,175 +595,175 @@
       <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>700</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>26</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>31</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>36</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>46</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>51</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>56</v>
-      </c>
-      <c r="K2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>500</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>32</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>37</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>42</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>47</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>52</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>57</v>
-      </c>
-      <c r="K3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4">
+        <v>121</v>
+      </c>
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>33</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>38</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>43</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>48</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>53</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>58</v>
-      </c>
-      <c r="K4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5">
+        <v>264</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>34</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>39</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>44</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>49</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>54</v>
       </c>
-      <c r="J5" t="s">
-        <v>59</v>
-      </c>
       <c r="K5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6">
+        <v>285</v>
+      </c>
+      <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>30</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>45</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>50</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>55</v>
       </c>
-      <c r="J6" t="s">
-        <v>60</v>
-      </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>